<commit_message>
Phase 5a/5b expanded: 18 SDTM domains (DV DS MH EG TU TR RS)
</commit_message>
<xml_diff>
--- a/acrf_metadata.xlsx
+++ b/acrf_metadata.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Domain'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Domain'!$A$1:$I$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -642,7 +642,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -675,7 +675,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -708,7 +708,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -741,7 +741,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -799,7 +799,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -857,7 +857,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -886,7 +886,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -919,7 +919,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -952,7 +952,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -1478,27 +1478,31 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>EXENDTC</t>
+          <t>DSCAT</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Date of Last Dose:</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
+          <t>Category: PROTOCOL MILESTONE DISPOSITION EVENT OTHER</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>DSCAT</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 5 of 8</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -1507,492 +1511,432 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>EXSTDTC</t>
+          <t>DSDECOD</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Date of First Dose:</t>
+          <t>Standardized Disposition Term:</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 5 of 8</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>AEACNOTH</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Other Action Taken:</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 4</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>DSSCAT</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Subcategory:</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>DSSCAT</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>AESDTH</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Led to Death?: Yes No</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 4</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DSSTDTC</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Date of Disposition:</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>AESHOSP</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Led to Hospitalization?: Yes No</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 4</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>DSTERM</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Disposition Event:</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>AETRTEM</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Treatment Emergent?: Yes No</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 4</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I38" s="3" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>EPOCH</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Epoch:</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>EPOCH</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>SUPPCM</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>CMINDOTH</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Other Indication:</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Page 4 of 4</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>DVCAT</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Category: MAJOR MINOR</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>DVCAT</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>SUPPCM</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>CMPREVFL</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Prior Medication?: Yes No</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Page 4 of 4</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DVDECOD</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Deviation Coded Term:</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>COMPLT</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Completed Study?: Yes No</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 4</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>DVSCAT</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Subcategory:</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>DVSCAT</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>DCSREAS</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Reason for Discontinuation:</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>DCSREAS</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 4</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>DVSTDTC</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Deviation Date:</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>EDUYRN</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Years of Education:</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 4</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>DVTERM</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Deviation Term:</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>SUPPVS</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>VSCLSIG</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Clinically Significant?: Yes No</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Page 2 of 4</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I44" s="3" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>EPOCH</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Epoch:</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>EPOCH</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>SUPPVS</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>VSFAST</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Fasting?: Yes No</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Page 2 of 4</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>EGDTC</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>ECG Date:</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>SUPPVS</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>VSLOC</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Location of Measurement:</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>LOC</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Page 2 of 4</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I46" s="3" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>EGEVAL</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Overall Interpretation: Normal Abnormal NCS Abnormal CS</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>NCSAB</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>VISIT</t>
+          <t>EGSTRESN</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Visit Name:</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>VISIT</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>Heart Rate (bpm):</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>EGTESTCD=HR</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -2001,27 +1945,31 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>VSDTC</t>
+          <t>EGSTRESN</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Visit Date:</t>
+          <t>PR Interval (msec):</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>EGTESTCD=PRINTR</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2030,31 +1978,31 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>VSPOS</t>
+          <t>EGSTRESN</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Position: Sitting Standing Supine</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>POSITION</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+          <t>QRS Duration (msec):</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>EGTESTCD=QRSDUR</t>
+        </is>
+      </c>
       <c r="F49" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2063,31 +2011,31 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>EGSTRESN</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Systolic Blood Pressure (mmHg):</t>
+          <t>QT Interval (msec):</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>VSTESTCD=SYSBP</t>
+          <t>EGTESTCD=QTINT</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2096,31 +2044,31 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>EGSTRESN</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Diastolic Blood Pressure (mmHg):</t>
+          <t>QTcF (msec):</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>VSTESTCD=DIABP</t>
+          <t>EGTESTCD=QTCF</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -2129,31 +2077,31 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>VISIT</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Heart Rate (beats/min):</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=HR</t>
-        </is>
-      </c>
+          <t>Visit Name:</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2162,31 +2110,27 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>EXENDTC</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Temperature (C):</t>
+          <t>Date of Last Dose:</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=TEMP</t>
-        </is>
-      </c>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -2195,31 +2139,27 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>EXSTDTC</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Weight (kg):</t>
+          <t>Date of First Dose:</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=WEIGHT</t>
-        </is>
-      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -2228,38 +2168,1692 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>MHBODSYS</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Height (cm):</t>
+          <t>Body System:</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=HEIGHT</t>
-        </is>
-      </c>
+      <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 5 of 8</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr"/>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>MHCAT</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Category: General Surgical Family</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>MHCAT</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>MHDECOD</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Dictionary Coded Term:</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>MHENDTC</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>End Date:</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>MHENRF</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing?: Yes No</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>MHSTDTC</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Start Date:</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>MHTERM</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Condition (verbatim):</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Page 5 of 8</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>RSCAT</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Response Criteria: RECIST 1.1 iRECIST</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>RSCAT</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>RSDTC</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Assessment Date:</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>RSEVAL</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Overall Response:</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=OVRLRESP</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Target Lesion Response:</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=TRGRESP</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Non-Target Response:</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=NTRGRESP</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>New Lesion Status:</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=NEWLIND</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>SUPPAE</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>AEACNOTH</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Other Action Taken:</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Page 3 of 8</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>SUPPAE</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>AESDTH</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Led to Death?: Yes No</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr"/>
+      <c r="F70" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Page 3 of 8</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>SUPPAE</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>AESHOSP</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Led to Hospitalization?: Yes No</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Page 3 of 8</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>SUPPAE</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>AETRTEM</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Treatment Emergent?: Yes No</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr"/>
+      <c r="F72" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Page 3 of 8</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>SUPPCM</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>CMINDOTH</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Other Indication:</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr"/>
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Page 4 of 8</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>SUPPCM</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>CMPREVFL</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Prior Medication?: Yes No</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Page 4 of 8</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>COMPLT</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Completed Study?: Yes No</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 8</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>DCSREAS</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Reason for Discontinuation:</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>DCSREAS</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 8</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>EDUYRN</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Years of Education:</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr"/>
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 8</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>SUPPEG</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>EGCLSIG</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Clinically Significant?: Yes No</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr"/>
+      <c r="F78" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>RSBORRESP</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Best Overall Response: CR PR SD PD</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>RSRESP</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>RSCONFDTC</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Date of Confirmation:</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr"/>
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>RSCONFYN</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed Response?: Yes No</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr"/>
+      <c r="F81" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>VSCLSIG</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Clinically Significant?: Yes No</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr"/>
+      <c r="F82" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>VSFAST</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Fasting?: Yes No</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr"/>
+      <c r="F83" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>VSLOC</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Location of Measurement:</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>LOC</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr"/>
+      <c r="F84" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>TRDTC</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Measurement Date:</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>TREVAL</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>TRLNKID</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Linked Tumor ID:</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>TRSTRESN</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Longest Diameter (mm):</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>TRTESTCD=LDIAM</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>TRSTRESN</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Short Axis Diameter (mm):</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>TRTESTCD=SAXIS</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>TRSTRESN</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Sum of Diameters (mm):</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>TRTESTCD=SUMDIAM</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>TUDTC</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Assessment Date:</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>TUEVAL</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>TULAT</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Laterality: Left Right Bilateral</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>LAT</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>TULNKID</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Tumor ID:</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>TULOC</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Location:</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>LOC</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>TUMETHOD</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Method: CT MRI Physical Exam X-ray</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>METHOD</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Visit Name:</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>VSDTC</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Visit Date:</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>VSPOS</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Position: Sitting Standing Supine</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>POSITION</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Systolic Blood Pressure (mmHg):</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=SYSBP</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Diastolic Blood Pressure (mmHg):</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=DIABP</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Heart Rate (beats/min):</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr"/>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=HR</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Temperature (C):</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr"/>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=TEMP</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Weight (kg):</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=WEIGHT</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Height (cm):</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr"/>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=HEIGHT</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2270,7 +3864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2317,7 +3911,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 3 of 8</t>
         </is>
       </c>
     </row>
@@ -2337,7 +3931,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 4 of 8</t>
         </is>
       </c>
     </row>
@@ -2357,18 +3951,18 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -2377,118 +3971,298 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 5 of 8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>SUPPAE</t>
+          <t>DV</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SUPP</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Page 3 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>SUPPCM</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>SUPP</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Page 4 of 4</t>
+          <t>Page 6 of 8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>SUPPDM</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SUPP</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 4</t>
+          <t>Page 1 of 8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>SUPPVS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>SUPP</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Page 2 of 4</t>
+          <t>Page 5 of 8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>SUPPAE</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Page 3 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>SUPPCM</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Page 4 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Page 1 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>SUPPEG</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Page 6 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Page 8 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>SUPP</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Page 7 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>VS</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B19" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Page 2 of 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Page 2 of 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
-        <v>54</v>
+      <c r="B20" s="6" t="n">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add ADLB; LB in sample aCRF; domain-specific visit windows
</commit_message>
<xml_diff>
--- a/acrf_metadata.xlsx
+++ b/acrf_metadata.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Domain'!$A$1:$I$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'By Domain'!$A$1:$I$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -547,11 +547,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -576,11 +576,11 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -605,11 +605,11 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -638,11 +638,11 @@
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -671,11 +671,11 @@
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -704,11 +704,11 @@
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -737,11 +737,11 @@
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -766,11 +766,11 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -795,11 +795,11 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -824,11 +824,11 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -853,11 +853,11 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -882,11 +882,11 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -915,11 +915,11 @@
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -948,11 +948,11 @@
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -977,11 +977,11 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1006,11 +1006,11 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1039,11 +1039,11 @@
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1101,11 +1101,11 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1130,11 +1130,11 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -1498,11 +1498,11 @@
       </c>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -1527,11 +1527,11 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -1560,11 +1560,11 @@
       </c>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -1589,11 +1589,11 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -1618,11 +1618,11 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -1651,11 +1651,11 @@
       </c>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -1684,11 +1684,11 @@
       </c>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -1713,11 +1713,11 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -1746,11 +1746,11 @@
       </c>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -1775,11 +1775,11 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -1804,11 +1804,11 @@
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -1837,11 +1837,11 @@
       </c>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -1866,11 +1866,11 @@
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -1899,11 +1899,11 @@
       </c>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -1932,11 +1932,11 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -1965,11 +1965,11 @@
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -1998,11 +1998,11 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2031,11 +2031,11 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2064,11 +2064,11 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -2097,11 +2097,11 @@
       </c>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -2168,27 +2168,27 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>MHBODSYS</t>
+          <t>LBDTC</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Body System:</t>
+          <t>Collection Date:</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -2197,31 +2197,31 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>MHCAT</t>
+          <t>LBFAST</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Category: General Surgical Family</t>
+          <t>Fasting?: Yes No</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>MHCAT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -2230,27 +2230,31 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>MHDECOD</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Dictionary Coded Term:</t>
+          <t>Glucose (mmol/L):</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=GLUC</t>
+        </is>
+      </c>
       <c r="F57" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -2259,27 +2263,31 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>MHENDTC</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>End Date:</t>
+          <t>Creatinine (umol/L):</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=CREAT</t>
+        </is>
+      </c>
       <c r="F58" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -2288,31 +2296,31 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>MHENRF</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Ongoing?: Yes No</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr"/>
+          <t>ALT (U/L):</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=ALT</t>
+        </is>
+      </c>
       <c r="F59" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -2321,27 +2329,31 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>MHSTDTC</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Start Date:</t>
+          <t>AST (U/L):</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=AST</t>
+        </is>
+      </c>
       <c r="F60" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -2350,27 +2362,31 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>MHTERM</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Condition (verbatim):</t>
+          <t>Total Bilirubin (umol/L):</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=BILI</t>
+        </is>
+      </c>
       <c r="F61" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -2379,31 +2395,31 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>RSCAT</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Response Criteria: RECIST 1.1 iRECIST</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>RSCAT</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
+          <t>Hemoglobin (g/L):</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=HGB</t>
+        </is>
+      </c>
       <c r="F62" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -2412,27 +2428,31 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>RSDTC</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Assessment Date:</t>
+          <t>White Blood Cells (10^9/L):</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
-      <c r="E63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=WBC</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -2441,31 +2461,31 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>RSEVAL</t>
+          <t>LBSTRESN</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>EVAL</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
+          <t>Platelets (10^9/L):</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>LBTESTCD=PLAT</t>
+        </is>
+      </c>
       <c r="F64" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -2474,31 +2494,31 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>RSORRES</t>
+          <t>VISIT</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Overall Response:</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>RSTESTCD=OVRLRESP</t>
-        </is>
-      </c>
+          <t>Visit Name:</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -2507,31 +2527,27 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>RSORRES</t>
+          <t>MHBODSYS</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Target Lesion Response:</t>
+          <t>Body System:</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>RSTESTCD=TRGRESP</t>
-        </is>
-      </c>
+      <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -2540,31 +2556,31 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>RSORRES</t>
+          <t>MHCAT</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Non-Target Response:</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr"/>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>RSTESTCD=NTRGRESP</t>
-        </is>
-      </c>
+          <t>Category: General Surgical Family</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>MHCAT</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -2573,455 +2589,403 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>RSORRES</t>
+          <t>MHDECOD</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>New Lesion Status:</t>
+          <t>Dictionary Coded Term:</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>RSTESTCD=NEWLIND</t>
-        </is>
-      </c>
+      <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>AEACNOTH</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>Other Action Taken:</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="3" t="inlineStr"/>
-      <c r="F69" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 8</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>MHENDTC</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>End Date:</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 9</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>AESDTH</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>Led to Death?: Yes No</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>MHENRF</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing?: Yes No</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 8</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 9</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>AESHOSP</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>Led to Hospitalization?: Yes No</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 8</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I71" s="3" t="inlineStr"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>MHSTDTC</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Start Date:</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 9</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>SUPPAE</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>AETRTEM</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>Treatment Emergent?: Yes No</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr"/>
-      <c r="F72" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>Page 3 of 8</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I72" s="3" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>MHTERM</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Condition (verbatim):</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Page 6 of 9</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="3" t="inlineStr">
-        <is>
-          <t>SUPPCM</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>CMINDOTH</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>Other Indication:</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr"/>
-      <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G73" s="3" t="inlineStr">
-        <is>
-          <t>Page 4 of 8</t>
-        </is>
-      </c>
-      <c r="H73" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I73" s="3" t="inlineStr"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>RSCAT</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Response Criteria: RECIST 1.1 iRECIST</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>RSCAT</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>SUPPCM</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>CMPREVFL</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>Prior Medication?: Yes No</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr"/>
-      <c r="F74" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>Page 4 of 8</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I74" s="3" t="inlineStr"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>RSDTC</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Assessment Date:</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>COMPLT</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>Completed Study?: Yes No</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 8</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I75" s="3" t="inlineStr"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>RSEVAL</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>DCSREAS</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>Reason for Discontinuation:</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>DCSREAS</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 8</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I76" s="3" t="inlineStr"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Overall Response:</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=OVRLRESP</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="3" t="inlineStr">
-        <is>
-          <t>SUPPDM</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>EDUYRN</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>Years of Education:</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr"/>
-      <c r="E77" s="3" t="inlineStr"/>
-      <c r="F77" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>Page 1 of 8</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I77" s="3" t="inlineStr"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Target Lesion Response:</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=TRGRESP</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>SUPPEG</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>EGCLSIG</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>Clinically Significant?: Yes No</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr"/>
-      <c r="F78" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G78" s="3" t="inlineStr">
-        <is>
-          <t>Page 6 of 8</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I78" s="3" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Non-Target Response:</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=NTRGRESP</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>SUPPRS</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>RSBORRESP</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>Best Overall Response: CR PR SD PD</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>RSRESP</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr"/>
-      <c r="F79" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="G79" s="3" t="inlineStr">
-        <is>
-          <t>Page 8 of 8</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>RSORRES</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>New Lesion Status:</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>RSTESTCD=NEWLIND</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>SUPPRS</t>
+          <t>SUPPAE</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>RSCONFDTC</t>
+          <t>AEACNOTH</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Date of Confirmation:</t>
+          <t>Other Action Taken:</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr"/>
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
@@ -3034,17 +2998,17 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>SUPPRS</t>
+          <t>SUPPAE</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>RSCONFYN</t>
+          <t>AESDTH</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Confirmed Response?: Yes No</t>
+          <t>Led to Death?: Yes No</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -3054,11 +3018,11 @@
       </c>
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
@@ -3071,17 +3035,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>SUPPVS</t>
+          <t>SUPPAE</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>VSCLSIG</t>
+          <t>AESHOSP</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Clinically Significant?: Yes No</t>
+          <t>Led to Hospitalization?: Yes No</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -3091,11 +3055,11 @@
       </c>
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
@@ -3108,17 +3072,17 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>SUPPVS</t>
+          <t>SUPPAE</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>VSFAST</t>
+          <t>AETRTEM</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Fasting?: Yes No</t>
+          <t>Treatment Emergent?: Yes No</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -3128,11 +3092,11 @@
       </c>
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
@@ -3145,448 +3109,496 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>SUPPVS</t>
+          <t>SUPPCM</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>VSLOC</t>
+          <t>CMINDOTH</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Location of Measurement:</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>LOC</t>
-        </is>
-      </c>
+          <t>Other Indication:</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr"/>
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Page 5 of 9</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>SUPPCM</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>CMPREVFL</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Prior Medication?: Yes No</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Page 5 of 9</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>COMPLT</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Completed Study?: Yes No</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 9</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>DCSREAS</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Reason for Discontinuation:</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>DCSREAS</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 9</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>SUPPDM</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>EDUYRN</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Years of Education:</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr"/>
+      <c r="E88" s="3" t="inlineStr"/>
+      <c r="F88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Page 1 of 9</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>SUPPEG</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>EGCLSIG</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Clinically Significant?: Yes No</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr"/>
+      <c r="F89" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>Page 7 of 9</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>SUPPLB</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>LBCLSIG</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Clinically Significant?: Yes No</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr"/>
+      <c r="F90" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>Page 3 of 9</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>RSBORRESP</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Best Overall Response: CR PR SD PD</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>RSRESP</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>RSCONFDTC</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Date of Confirmation:</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr"/>
+      <c r="F92" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>SUPPRS</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>RSCONFYN</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed Response?: Yes No</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>Page 9 of 9</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>VSCLSIG</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Clinically Significant?: Yes No</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G84" s="3" t="inlineStr">
-        <is>
-          <t>Page 2 of 8</t>
-        </is>
-      </c>
-      <c r="H84" s="3" t="inlineStr">
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I84" s="3" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>TRDTC</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Measurement Date:</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr"/>
-      <c r="E85" s="2" t="inlineStr"/>
-      <c r="F85" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr"/>
-      <c r="I85" s="2" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>TREVAL</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>EVAL</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G86" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr"/>
-      <c r="I86" s="2" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>TRLNKID</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>Linked Tumor ID:</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr"/>
-      <c r="E87" s="2" t="inlineStr"/>
-      <c r="F87" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>TRSTRESN</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>Longest Diameter (mm):</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr"/>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>TRTESTCD=LDIAM</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr"/>
-      <c r="I88" s="2" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>TRSTRESN</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>Short Axis Diameter (mm):</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr"/>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>TRTESTCD=SAXIS</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G89" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>TRSTRESN</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>Sum of Diameters (mm):</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr"/>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>TRTESTCD=SUMDIAM</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>TUDTC</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>Assessment Date:</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr"/>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr"/>
-      <c r="I91" s="2" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>TUEVAL</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>EVAL</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr"/>
-      <c r="F92" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="inlineStr"/>
-      <c r="I92" s="2" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>TULAT</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>Laterality: Left Right Bilateral</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>LAT</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr"/>
-      <c r="F93" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G93" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H93" s="2" t="inlineStr"/>
-      <c r="I93" s="2" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>TULNKID</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>Tumor ID:</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr"/>
-      <c r="E94" s="2" t="inlineStr"/>
-      <c r="F94" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr"/>
-      <c r="I94" s="2" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>TULOC</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>Tumor Location:</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>VSFAST</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Fasting?: Yes No</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr"/>
+      <c r="F95" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>SUPPVS</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>VSLOC</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Location of Measurement:</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>LOC</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr"/>
-      <c r="F95" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G95" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H95" s="2" t="inlineStr"/>
-      <c r="I95" s="2" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>TU</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>TUMETHOD</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>Method: CT MRI Physical Exam X-ray</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>METHOD</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr"/>
-      <c r="F96" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>Page 7 of 8</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr"/>
-      <c r="I96" s="2" t="inlineStr"/>
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>VISIT</t>
+          <t>TRDTC</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Visit Name:</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>VISIT</t>
-        </is>
-      </c>
+          <t>Measurement Date:</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr"/>
@@ -3595,27 +3607,31 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>VSDTC</t>
+          <t>TREVAL</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Visit Date:</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr"/>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr"/>
@@ -3624,31 +3640,27 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>VSPOS</t>
+          <t>TRLNKID</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Position: Sitting Standing Supine</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>POSITION</t>
-        </is>
-      </c>
+          <t>Linked Tumor ID:</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -3657,31 +3669,31 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TRSTRESN</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Systolic Blood Pressure (mmHg):</t>
+          <t>Longest Diameter (mm):</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr"/>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>VSTESTCD=SYSBP</t>
+          <t>TRTESTCD=LDIAM</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -3690,31 +3702,31 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TRSTRESN</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Diastolic Blood Pressure (mmHg):</t>
+          <t>Short Axis Diameter (mm):</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr"/>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>VSTESTCD=DIABP</t>
+          <t>TRTESTCD=SAXIS</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
@@ -3723,31 +3735,31 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TRSTRESN</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Heart Rate (beats/min):</t>
+          <t>Sum of Diameters (mm):</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>VSTESTCD=HR</t>
+          <t>TRTESTCD=SUMDIAM</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr"/>
@@ -3756,31 +3768,27 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TUDTC</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Temperature (C):</t>
+          <t>Assessment Date:</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr"/>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=TEMP</t>
-        </is>
-      </c>
+      <c r="E103" s="2" t="inlineStr"/>
       <c r="F103" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -3789,31 +3797,31 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TUEVAL</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Weight (kg):</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr"/>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=WEIGHT</t>
-        </is>
-      </c>
+          <t>Evaluator: INVESTIGATOR INDEPENDENT ASSESSOR</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>EVAL</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr"/>
@@ -3822,38 +3830,426 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>VS</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>VSSTRESN</t>
+          <t>TULAT</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Height (cm):</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr"/>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>VSTESTCD=HEIGHT</t>
-        </is>
-      </c>
+          <t>Laterality: Left Right Bilateral</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>LAT</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 8 of 9</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr"/>
       <c r="I105" s="2" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>TULNKID</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Tumor ID:</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 9</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>TULOC</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Tumor Location:</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>LOC</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 9</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>TUMETHOD</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Method: CT MRI Physical Exam X-ray</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>METHOD</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Page 8 of 9</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Visit Name:</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>VISIT</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr"/>
+      <c r="I109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>VSDTC</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Visit Date:</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>VSPOS</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Position: Sitting Standing Supine</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>POSITION</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr"/>
+      <c r="I111" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Systolic Blood Pressure (mmHg):</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr"/>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=SYSBP</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Diastolic Blood Pressure (mmHg):</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr"/>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=DIABP</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr"/>
+      <c r="I113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Heart Rate (beats/min):</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr"/>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=HR</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Temperature (C):</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr"/>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=TEMP</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr"/>
+      <c r="I115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Weight (kg):</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr"/>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=WEIGHT</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>VSSTRESN</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Height (cm):</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr"/>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>VSTESTCD=HEIGHT</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr"/>
+      <c r="I117" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I105"/>
+  <autoFilter ref="A1:I117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3864,7 +4260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3911,7 +4307,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
     </row>
@@ -3931,7 +4327,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
     </row>
@@ -3951,7 +4347,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
     </row>
@@ -3971,7 +4367,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
     </row>
@@ -3991,7 +4387,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4407,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
     </row>
@@ -4031,18 +4427,18 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
@@ -4051,14 +4447,14 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Page 5 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -4071,38 +4467,38 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 6 of 9</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>SUPPAE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>SUPP</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Page 3 of 8</t>
+          <t>Page 9 of 9</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>SUPPCM</t>
+          <t>SUPPAE</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -4111,18 +4507,18 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Page 4 of 8</t>
+          <t>Page 4 of 9</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>SUPPDM</t>
+          <t>SUPPCM</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -4131,18 +4527,18 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Page 1 of 8</t>
+          <t>Page 5 of 9</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>SUPPEG</t>
+          <t>SUPPDM</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -4151,18 +4547,18 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Page 6 of 8</t>
+          <t>Page 1 of 9</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>SUPPRS</t>
+          <t>SUPPEG</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -4171,18 +4567,18 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Page 8 of 8</t>
+          <t>Page 7 of 9</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>SUPPVS</t>
+          <t>SUPPLB</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -4191,78 +4587,118 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Page 2 of 8</t>
+          <t>Page 3 of 9</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>SUPPRS</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>SUPP</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Page 7 of 8</t>
+          <t>Page 9 of 9</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>SUPPVS</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>SUPP</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Page 7 of 8</t>
+          <t>Page 2 of 9</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Page 8 of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>TU</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Page 8 of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>VS</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Page 2 of 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Page 2 of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
-        <v>104</v>
+      <c r="B22" s="6" t="n">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>